<commit_message>
Add questions: EVP Brand
</commit_message>
<xml_diff>
--- a/surveys/evp-brand/questions.xlsx
+++ b/surveys/evp-brand/questions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tillamook-my.sharepoint.com/personal/mhaight_tillamook_com/Documents/InterviewGuidesExe/InterviewGuidesExe/surveys/evp-brand/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_9D71ECEA8B1CDAF8E8E638153A53DA92D1B991C2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E19B0A6-9518-43FF-A1D8-868301D48786}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="11_9D71ECEA8B1CDAF8E8E638153A53DA92D1B991C2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6628EC35-A014-468B-A572-18C643D73DAD}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Setup" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="41">
   <si>
     <t>EVP Brand</t>
   </si>
@@ -47,34 +47,103 @@
     <t>Skill Based</t>
   </si>
   <si>
-    <t>How does your experience relate to this position?</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Walk me through a complex project you completed.</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>Competency</t>
   </si>
   <si>
-    <t>Describe a time you had to make a difficult decision quickly.</t>
-  </si>
-  <si>
-    <t>Tell me about a challenge you faced and how you resolved it.</t>
-  </si>
-  <si>
     <t>Shared Values</t>
   </si>
   <si>
-    <t>Which of our Shared Values resonates most with you and why?</t>
-  </si>
-  <si>
-    <t>Tell me about a time you demonstrated one of our core values at work.</t>
+    <t>No Interview Guide</t>
+  </si>
+  <si>
+    <t>index.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tell us about a time when you transformed an organization or function while continuing to deliver results. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tell us about a time you influenced a major strategic decision outside your direct authority. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">As an ELT member, how do you ensure enterprise priorities are balanced with functional priorities? </t>
+  </si>
+  <si>
+    <t>If selected, what would be your priorities during your first 100 days?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Many brands talk about purpose. How do you ensure purpose and values remain authentic and create business value? </t>
+  </si>
+  <si>
+    <t>What are the biggest threats to consumer trust for a modern food company, and how should leaders prepare for them?</t>
+  </si>
+  <si>
+    <t>Tell us about a situation where making the right decision was unpopular but necessary for the long-term health of the brand.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What draws you to Tillamook specifically, and why is this role compelling at this stage of your career? </t>
+  </si>
+  <si>
+    <t>Three years from now, what outcomes would need to be true for you to consider your tenure a success?</t>
+  </si>
+  <si>
+    <t>What role should an executive brand leader play in shaping organizational culture?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How do you define the role of a brand in driving enterprise value beyond marketing? Can you share an example where brand strategy directly influenced business strategy? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">How do you stay ahead of shifts in consumer behavior and translate emerging trends into business opportunities? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">What metrics do you use to determine whether brand investments are creating enterprise value? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">If you inherited a constrained budget, how would you determine where to invest and where to pull back? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">What must Tillamook do to maintain premium positioning while competing in an increasingly value-focused marketplace? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">What role should brand play in strengthening strategic retailer relationships? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Describe a time when you successfully expanded a brand into adjacent categories or channels. </t>
+  </si>
+  <si>
+    <t>What has been your most successful partnership with commercial, operations, or supply chain leaders?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Based on what you've learned about Tillamook, where do you see the biggest opportunities for growth over the next five years? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Describe the strongest leadership team you've built. What were the key attributes and how did you develop them? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">How do you assess leadership potential and succession readiness within your organization? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">What have you done to build stronger marketing, creative, or commercial capabilities within your organization? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tell us about a time you led in an environment with competing stakeholder interests. How did you build alignment? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Describe a situation where healthy debate led to a better business outcome. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">What specific actions have you taken to create an environment where diverse perspectives are actively sought and valued? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">How do you respond when a team member challenges your perspective or recommendation? </t>
+  </si>
+  <si>
+    <t>How have you measured or improved employee engagement, inclusion, or team effectiveness within your organization?</t>
+  </si>
+  <si>
+    <t>Tillamook is a beloved regional brand that has become a national player. What are the greatest risks when scaling a trusted legacy brand?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How would you preserve Tillamook's farmer-owned cooperative identity while accelerating national growth? </t>
   </si>
 </sst>
 </file>
@@ -493,7 +562,14 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A4:B4"/>
@@ -505,7 +581,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -529,10 +605,7 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -540,58 +613,227 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" t="s">
         <v>15</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>8</v>
+      </c>
+      <c r="B19" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>8</v>
+      </c>
+      <c r="B20" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>8</v>
+      </c>
+      <c r="B23" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" t="s">
         <v>17</v>
       </c>
-      <c r="C7" t="s">
-        <v>11</v>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>9</v>
+      </c>
+      <c r="B28" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>9</v>
+      </c>
+      <c r="B29" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>9</v>
+      </c>
+      <c r="B30" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" sqref="A2:A500" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Skill Based,Competency,Shared Values"</formula1>
     </dataValidation>

</xml_diff>